<commit_message>
Deleted 0.01 contrast, added 0.025
</commit_message>
<xml_diff>
--- a/Conditions_parameters.xlsx
+++ b/Conditions_parameters.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Asus\Documents\H-IBL.TaskPretest\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{43B99C88-5FC6-4741-AF1C-6CAF2C3C7936}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8BCAB7BC-DD42-4769-B809-29CE4AF09F8C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -44,7 +44,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="135" uniqueCount="24">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="119" uniqueCount="23">
   <si>
     <t>position</t>
   </si>
@@ -100,12 +100,6 @@
     <t>0.16</t>
   </si>
   <si>
-    <t>0.32</t>
-  </si>
-  <si>
-    <t>0.01</t>
-  </si>
-  <si>
     <t>0.02</t>
   </si>
   <si>
@@ -116,6 +110,9 @@
   </si>
   <si>
     <t>(-30,0)</t>
+  </si>
+  <si>
+    <t>0.025</t>
   </si>
 </sst>
 </file>
@@ -439,7 +436,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:N17"/>
+  <dimension ref="A1:N15"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="8" max="8" width="9.7109375" customWidth="1"/>
@@ -482,7 +479,7 @@
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="B2">
         <v>0</v>
@@ -517,7 +514,7 @@
     </row>
     <row r="3" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="B3">
         <v>0</v>
@@ -552,10 +549,10 @@
     </row>
     <row r="4" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="B4" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C4" t="s">
         <v>11</v>
@@ -587,10 +584,10 @@
     </row>
     <row r="5" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="B5" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C5" t="s">
         <v>11</v>
@@ -622,10 +619,10 @@
     </row>
     <row r="6" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="B6" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="C6" t="s">
         <v>11</v>
@@ -657,10 +654,10 @@
     </row>
     <row r="7" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="B7" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="C7" t="s">
         <v>11</v>
@@ -692,10 +689,10 @@
     </row>
     <row r="8" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="B8" t="s">
-        <v>21</v>
+        <v>8</v>
       </c>
       <c r="C8" t="s">
         <v>11</v>
@@ -727,10 +724,10 @@
     </row>
     <row r="9" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="B9" t="s">
-        <v>21</v>
+        <v>8</v>
       </c>
       <c r="C9" t="s">
         <v>11</v>
@@ -762,10 +759,10 @@
     </row>
     <row r="10" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="B10" t="s">
-        <v>8</v>
+        <v>17</v>
       </c>
       <c r="C10" t="s">
         <v>11</v>
@@ -797,10 +794,10 @@
     </row>
     <row r="11" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="B11" t="s">
-        <v>8</v>
+        <v>17</v>
       </c>
       <c r="C11" t="s">
         <v>11</v>
@@ -832,10 +829,10 @@
     </row>
     <row r="12" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
+        <v>20</v>
+      </c>
+      <c r="B12" t="s">
         <v>22</v>
-      </c>
-      <c r="B12" t="s">
-        <v>17</v>
       </c>
       <c r="C12" t="s">
         <v>11</v>
@@ -867,10 +864,10 @@
     </row>
     <row r="13" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="B13" t="s">
-        <v>17</v>
+        <v>22</v>
       </c>
       <c r="C13" t="s">
         <v>11</v>
@@ -900,12 +897,12 @@
         <v>8</v>
       </c>
     </row>
-    <row r="14" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:14" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>22</v>
-      </c>
-      <c r="B14" t="s">
-        <v>18</v>
+        <v>20</v>
+      </c>
+      <c r="B14">
+        <v>1</v>
       </c>
       <c r="C14" t="s">
         <v>11</v>
@@ -937,10 +934,10 @@
     </row>
     <row r="15" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>23</v>
-      </c>
-      <c r="B15" t="s">
-        <v>18</v>
+        <v>21</v>
+      </c>
+      <c r="B15">
+        <v>1</v>
       </c>
       <c r="C15" t="s">
         <v>11</v>
@@ -967,76 +964,6 @@
         <v>9</v>
       </c>
       <c r="N15" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="16" spans="1:14" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A16" t="s">
-        <v>22</v>
-      </c>
-      <c r="B16">
-        <v>1</v>
-      </c>
-      <c r="C16" t="s">
-        <v>11</v>
-      </c>
-      <c r="D16" t="s">
-        <v>16</v>
-      </c>
-      <c r="E16">
-        <v>3</v>
-      </c>
-      <c r="F16">
-        <v>1</v>
-      </c>
-      <c r="G16">
-        <v>0</v>
-      </c>
-      <c r="H16" t="s">
-        <v>3</v>
-      </c>
-      <c r="L16" t="s">
-        <v>7</v>
-      </c>
-      <c r="M16" t="s">
-        <v>9</v>
-      </c>
-      <c r="N16" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="17" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A17" t="s">
-        <v>23</v>
-      </c>
-      <c r="B17">
-        <v>1</v>
-      </c>
-      <c r="C17" t="s">
-        <v>11</v>
-      </c>
-      <c r="D17" t="s">
-        <v>16</v>
-      </c>
-      <c r="E17">
-        <v>3</v>
-      </c>
-      <c r="F17">
-        <v>1</v>
-      </c>
-      <c r="G17">
-        <v>0</v>
-      </c>
-      <c r="H17" t="s">
-        <v>3</v>
-      </c>
-      <c r="L17" t="s">
-        <v>7</v>
-      </c>
-      <c r="M17" t="s">
-        <v>9</v>
-      </c>
-      <c r="N17" t="s">
         <v>8</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Contrasts: 0%, 1%, 2%, 2.5%, 4%, 8%
</commit_message>
<xml_diff>
--- a/Conditions_parameters.xlsx
+++ b/Conditions_parameters.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Asus\Documents\H-IBL.TaskPretest\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8BCAB7BC-DD42-4769-B809-29CE4AF09F8C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{83B9A262-A81D-4E62-82A0-503AD817CC91}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28920" yWindow="-2790" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -97,9 +97,6 @@
     <t>gauss</t>
   </si>
   <si>
-    <t>0.16</t>
-  </si>
-  <si>
     <t>0.02</t>
   </si>
   <si>
@@ -113,6 +110,9 @@
   </si>
   <si>
     <t>0.025</t>
+  </si>
+  <si>
+    <t>0.01</t>
   </si>
 </sst>
 </file>
@@ -479,7 +479,7 @@
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B2">
         <v>0</v>
@@ -514,7 +514,7 @@
     </row>
     <row r="3" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B3">
         <v>0</v>
@@ -549,10 +549,10 @@
     </row>
     <row r="4" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B4" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C4" t="s">
         <v>11</v>
@@ -584,10 +584,10 @@
     </row>
     <row r="5" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B5" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C5" t="s">
         <v>11</v>
@@ -619,10 +619,10 @@
     </row>
     <row r="6" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B6" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C6" t="s">
         <v>11</v>
@@ -654,10 +654,10 @@
     </row>
     <row r="7" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B7" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C7" t="s">
         <v>11</v>
@@ -689,7 +689,7 @@
     </row>
     <row r="8" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B8" t="s">
         <v>8</v>
@@ -724,7 +724,7 @@
     </row>
     <row r="9" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B9" t="s">
         <v>8</v>
@@ -759,10 +759,10 @@
     </row>
     <row r="10" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B10" t="s">
-        <v>17</v>
+        <v>22</v>
       </c>
       <c r="C10" t="s">
         <v>11</v>
@@ -794,10 +794,10 @@
     </row>
     <row r="11" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B11" t="s">
-        <v>17</v>
+        <v>22</v>
       </c>
       <c r="C11" t="s">
         <v>11</v>
@@ -829,10 +829,10 @@
     </row>
     <row r="12" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B12" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="C12" t="s">
         <v>11</v>
@@ -864,10 +864,10 @@
     </row>
     <row r="13" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
+        <v>20</v>
+      </c>
+      <c r="B13" t="s">
         <v>21</v>
-      </c>
-      <c r="B13" t="s">
-        <v>22</v>
       </c>
       <c r="C13" t="s">
         <v>11</v>
@@ -899,7 +899,7 @@
     </row>
     <row r="14" spans="1:14" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B14">
         <v>1</v>
@@ -934,7 +934,7 @@
     </row>
     <row r="15" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B15">
         <v>1</v>

</xml_diff>